<commit_message>
Project Implementation Timeline Ghant Chart
</commit_message>
<xml_diff>
--- a/source/MySEProject/Documentation/Project Implementation Timeline Ghant Chart.xlsx
+++ b/source/MySEProject/Documentation/Project Implementation Timeline Ghant Chart.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SE Project\neocortexapi\source\MySEProject\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -201,13 +201,13 @@
     <t xml:space="preserve">Project testing and initial final project deployement </t>
   </si>
   <si>
-    <t xml:space="preserve">Verify bugs and final final project deployement </t>
-  </si>
-  <si>
     <t xml:space="preserve">Write documentations </t>
   </si>
   <si>
     <t>Finalise and submission</t>
+  </si>
+  <si>
+    <t>Verify bugs and final final Project Deployement</t>
   </si>
 </sst>
 </file>
@@ -957,6 +957,63 @@
     <xf numFmtId="9" fontId="5" fillId="8" borderId="25" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="26" fillId="7" borderId="14" xfId="3" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="2" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="3" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="7" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="7" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="4" borderId="1" xfId="8" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="4" borderId="2" xfId="8" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="4" borderId="4" xfId="8" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="26" fillId="4" borderId="5" xfId="9" applyNumberFormat="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="26" fillId="4" borderId="6" xfId="9" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="4" borderId="7" xfId="8" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="4" borderId="8" xfId="8" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="4" borderId="9" xfId="8" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="9" borderId="16" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
@@ -974,63 +1031,6 @@
     </xf>
     <xf numFmtId="165" fontId="0" fillId="9" borderId="17" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="2" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="3" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="7" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="7" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="4" borderId="1" xfId="8" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="4" borderId="2" xfId="8" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="4" borderId="4" xfId="8" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="26" fillId="4" borderId="5" xfId="9" applyNumberFormat="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="26" fillId="4" borderId="6" xfId="9" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="4" borderId="7" xfId="8" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="4" borderId="8" xfId="8" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="4" borderId="9" xfId="8" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="26" fillId="7" borderId="14" xfId="3" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="11">
@@ -1046,157 +1046,7 @@
     <cellStyle name="Title" xfId="5" builtinId="15"/>
     <cellStyle name="zHiddenText" xfId="10"/>
   </cellStyles>
-  <dxfs count="31">
-    <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FFC00000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFC00000"/>
-        </right>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="0" tint="-0.34998626667073579"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="0" tint="-0.34998626667073579"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FFC00000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFC00000"/>
-        </right>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FFC00000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFC00000"/>
-        </right>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="0" tint="-0.34998626667073579"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="0" tint="-0.34998626667073579"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="0" tint="-0.34998626667073579"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FFC00000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFC00000"/>
-        </right>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FFC00000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFC00000"/>
-        </right>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FFC00000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFC00000"/>
-        </right>
-      </border>
-    </dxf>
+  <dxfs count="16">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1242,6 +1092,16 @@
           <bgColor theme="0" tint="-0.34998626667073579"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FFC00000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFC00000"/>
+        </right>
+      </border>
     </dxf>
     <dxf>
       <border>
@@ -1349,15 +1209,15 @@
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="ToDoList" pivot="0" count="9">
-      <tableStyleElement type="wholeTable" dxfId="30"/>
-      <tableStyleElement type="headerRow" dxfId="29"/>
-      <tableStyleElement type="totalRow" dxfId="28"/>
-      <tableStyleElement type="firstColumn" dxfId="27"/>
-      <tableStyleElement type="lastColumn" dxfId="26"/>
-      <tableStyleElement type="firstRowStripe" dxfId="25"/>
-      <tableStyleElement type="secondRowStripe" dxfId="24"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="23"/>
-      <tableStyleElement type="secondColumnStripe" dxfId="22"/>
+      <tableStyleElement type="wholeTable" dxfId="15"/>
+      <tableStyleElement type="headerRow" dxfId="14"/>
+      <tableStyleElement type="totalRow" dxfId="13"/>
+      <tableStyleElement type="firstColumn" dxfId="12"/>
+      <tableStyleElement type="lastColumn" dxfId="11"/>
+      <tableStyleElement type="firstRowStripe" dxfId="10"/>
+      <tableStyleElement type="secondRowStripe" dxfId="9"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="8"/>
+      <tableStyleElement type="secondColumnStripe" dxfId="7"/>
     </tableStyle>
   </tableStyles>
   <colors>
@@ -1711,7 +1571,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:FT16"/>
+  <dimension ref="A1:DB16"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="30" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="2.54296875" style="14" customWidth="1"/>
@@ -1737,13 +1597,13 @@
   <sheetData>
     <row r="1" spans="1:106" ht="30" customHeight="1" thickBot="1">
       <c r="A1" s="16"/>
-      <c r="B1" s="59" t="s">
+      <c r="B1" s="56" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="60"/>
-      <c r="D1" s="60"/>
-      <c r="E1" s="60"/>
-      <c r="F1" s="61"/>
+      <c r="C1" s="57"/>
+      <c r="D1" s="57"/>
+      <c r="E1" s="57"/>
+      <c r="F1" s="58"/>
       <c r="H1" s="5"/>
       <c r="I1" s="36"/>
     </row>
@@ -1751,180 +1611,180 @@
       <c r="A2" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="62" t="s">
+      <c r="B2" s="59" t="s">
         <v>33</v>
       </c>
-      <c r="C2" s="63"/>
-      <c r="D2" s="63"/>
-      <c r="E2" s="63"/>
-      <c r="F2" s="64"/>
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="60"/>
+      <c r="F2" s="61"/>
       <c r="I2" s="37"/>
     </row>
     <row r="3" spans="1:106" ht="30" customHeight="1" thickBot="1">
-      <c r="B3" s="65" t="s">
+      <c r="B3" s="62" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="66"/>
-      <c r="D3" s="67"/>
-      <c r="E3" s="68">
+      <c r="C3" s="63"/>
+      <c r="D3" s="64"/>
+      <c r="E3" s="65">
         <f>DATE(2025,1,1)</f>
         <v>45658</v>
       </c>
-      <c r="F3" s="69"/>
+      <c r="F3" s="66"/>
     </row>
     <row r="4" spans="1:106" ht="30" customHeight="1" thickBot="1">
       <c r="A4" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="70" t="s">
+      <c r="B4" s="67" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="71"/>
-      <c r="D4" s="72"/>
-      <c r="E4" s="73">
+      <c r="C4" s="68"/>
+      <c r="D4" s="69"/>
+      <c r="E4" s="70">
         <v>1</v>
       </c>
-      <c r="F4" s="74"/>
-      <c r="I4" s="53">
+      <c r="F4" s="71"/>
+      <c r="I4" s="72">
         <f>I5</f>
         <v>45656</v>
       </c>
-      <c r="J4" s="54"/>
-      <c r="K4" s="54"/>
-      <c r="L4" s="54"/>
-      <c r="M4" s="54"/>
-      <c r="N4" s="54"/>
-      <c r="O4" s="55"/>
-      <c r="P4" s="53">
+      <c r="J4" s="73"/>
+      <c r="K4" s="73"/>
+      <c r="L4" s="73"/>
+      <c r="M4" s="73"/>
+      <c r="N4" s="73"/>
+      <c r="O4" s="74"/>
+      <c r="P4" s="72">
         <f>P5</f>
         <v>45663</v>
       </c>
-      <c r="Q4" s="54"/>
-      <c r="R4" s="54"/>
-      <c r="S4" s="54"/>
-      <c r="T4" s="54"/>
-      <c r="U4" s="54"/>
-      <c r="V4" s="55"/>
-      <c r="W4" s="53">
+      <c r="Q4" s="73"/>
+      <c r="R4" s="73"/>
+      <c r="S4" s="73"/>
+      <c r="T4" s="73"/>
+      <c r="U4" s="73"/>
+      <c r="V4" s="74"/>
+      <c r="W4" s="72">
         <f>W5</f>
         <v>45670</v>
       </c>
-      <c r="X4" s="54"/>
-      <c r="Y4" s="54"/>
-      <c r="Z4" s="54"/>
-      <c r="AA4" s="54"/>
-      <c r="AB4" s="54"/>
-      <c r="AC4" s="55"/>
-      <c r="AD4" s="53">
+      <c r="X4" s="73"/>
+      <c r="Y4" s="73"/>
+      <c r="Z4" s="73"/>
+      <c r="AA4" s="73"/>
+      <c r="AB4" s="73"/>
+      <c r="AC4" s="74"/>
+      <c r="AD4" s="72">
         <f>AD5</f>
         <v>45677</v>
       </c>
-      <c r="AE4" s="54"/>
-      <c r="AF4" s="54"/>
-      <c r="AG4" s="54"/>
-      <c r="AH4" s="54"/>
-      <c r="AI4" s="54"/>
-      <c r="AJ4" s="55"/>
-      <c r="AK4" s="53">
+      <c r="AE4" s="73"/>
+      <c r="AF4" s="73"/>
+      <c r="AG4" s="73"/>
+      <c r="AH4" s="73"/>
+      <c r="AI4" s="73"/>
+      <c r="AJ4" s="74"/>
+      <c r="AK4" s="72">
         <f>AK5</f>
         <v>45684</v>
       </c>
-      <c r="AL4" s="54"/>
-      <c r="AM4" s="54"/>
-      <c r="AN4" s="54"/>
-      <c r="AO4" s="54"/>
-      <c r="AP4" s="54"/>
-      <c r="AQ4" s="55"/>
-      <c r="AR4" s="53">
+      <c r="AL4" s="73"/>
+      <c r="AM4" s="73"/>
+      <c r="AN4" s="73"/>
+      <c r="AO4" s="73"/>
+      <c r="AP4" s="73"/>
+      <c r="AQ4" s="74"/>
+      <c r="AR4" s="72">
         <f>AR5</f>
         <v>45691</v>
       </c>
-      <c r="AS4" s="54"/>
-      <c r="AT4" s="54"/>
-      <c r="AU4" s="54"/>
-      <c r="AV4" s="54"/>
-      <c r="AW4" s="54"/>
-      <c r="AX4" s="55"/>
-      <c r="AY4" s="53">
+      <c r="AS4" s="73"/>
+      <c r="AT4" s="73"/>
+      <c r="AU4" s="73"/>
+      <c r="AV4" s="73"/>
+      <c r="AW4" s="73"/>
+      <c r="AX4" s="74"/>
+      <c r="AY4" s="72">
         <f>AY5</f>
         <v>45698</v>
       </c>
-      <c r="AZ4" s="54"/>
-      <c r="BA4" s="54"/>
-      <c r="BB4" s="54"/>
-      <c r="BC4" s="54"/>
-      <c r="BD4" s="54"/>
-      <c r="BE4" s="55"/>
-      <c r="BF4" s="53">
+      <c r="AZ4" s="73"/>
+      <c r="BA4" s="73"/>
+      <c r="BB4" s="73"/>
+      <c r="BC4" s="73"/>
+      <c r="BD4" s="73"/>
+      <c r="BE4" s="74"/>
+      <c r="BF4" s="72">
         <f>BF5</f>
         <v>45705</v>
       </c>
-      <c r="BG4" s="54"/>
-      <c r="BH4" s="54"/>
-      <c r="BI4" s="54"/>
-      <c r="BJ4" s="54"/>
-      <c r="BK4" s="54"/>
-      <c r="BL4" s="55"/>
-      <c r="BM4" s="53">
+      <c r="BG4" s="73"/>
+      <c r="BH4" s="73"/>
+      <c r="BI4" s="73"/>
+      <c r="BJ4" s="73"/>
+      <c r="BK4" s="73"/>
+      <c r="BL4" s="74"/>
+      <c r="BM4" s="72">
         <f>BM5</f>
         <v>45712</v>
       </c>
-      <c r="BN4" s="54"/>
-      <c r="BO4" s="54"/>
-      <c r="BP4" s="54"/>
-      <c r="BQ4" s="54"/>
-      <c r="BR4" s="54"/>
-      <c r="BS4" s="55"/>
-      <c r="BT4" s="56">
+      <c r="BN4" s="73"/>
+      <c r="BO4" s="73"/>
+      <c r="BP4" s="73"/>
+      <c r="BQ4" s="73"/>
+      <c r="BR4" s="73"/>
+      <c r="BS4" s="74"/>
+      <c r="BT4" s="75">
         <f>BT5</f>
         <v>45719</v>
       </c>
-      <c r="BU4" s="57"/>
-      <c r="BV4" s="57"/>
-      <c r="BW4" s="57"/>
-      <c r="BX4" s="57"/>
-      <c r="BY4" s="57"/>
-      <c r="BZ4" s="58"/>
-      <c r="CA4" s="53">
+      <c r="BU4" s="76"/>
+      <c r="BV4" s="76"/>
+      <c r="BW4" s="76"/>
+      <c r="BX4" s="76"/>
+      <c r="BY4" s="76"/>
+      <c r="BZ4" s="77"/>
+      <c r="CA4" s="72">
         <f>CA5</f>
         <v>45726</v>
       </c>
-      <c r="CB4" s="54"/>
-      <c r="CC4" s="54"/>
-      <c r="CD4" s="54"/>
-      <c r="CE4" s="54"/>
-      <c r="CF4" s="54"/>
-      <c r="CG4" s="55"/>
-      <c r="CH4" s="53">
+      <c r="CB4" s="73"/>
+      <c r="CC4" s="73"/>
+      <c r="CD4" s="73"/>
+      <c r="CE4" s="73"/>
+      <c r="CF4" s="73"/>
+      <c r="CG4" s="74"/>
+      <c r="CH4" s="72">
         <f>CH5</f>
         <v>45733</v>
       </c>
-      <c r="CI4" s="54"/>
-      <c r="CJ4" s="54"/>
-      <c r="CK4" s="54"/>
-      <c r="CL4" s="54"/>
-      <c r="CM4" s="54"/>
-      <c r="CN4" s="55"/>
-      <c r="CO4" s="53">
+      <c r="CI4" s="73"/>
+      <c r="CJ4" s="73"/>
+      <c r="CK4" s="73"/>
+      <c r="CL4" s="73"/>
+      <c r="CM4" s="73"/>
+      <c r="CN4" s="74"/>
+      <c r="CO4" s="72">
         <f>CO5</f>
         <v>45740</v>
       </c>
-      <c r="CP4" s="54"/>
-      <c r="CQ4" s="54"/>
-      <c r="CR4" s="54"/>
-      <c r="CS4" s="54"/>
-      <c r="CT4" s="54"/>
-      <c r="CU4" s="55"/>
-      <c r="CV4" s="53">
+      <c r="CP4" s="73"/>
+      <c r="CQ4" s="73"/>
+      <c r="CR4" s="73"/>
+      <c r="CS4" s="73"/>
+      <c r="CT4" s="73"/>
+      <c r="CU4" s="74"/>
+      <c r="CV4" s="72">
         <f>CV5</f>
         <v>45747</v>
       </c>
-      <c r="CW4" s="54"/>
-      <c r="CX4" s="54"/>
-      <c r="CY4" s="54"/>
-      <c r="CZ4" s="54"/>
-      <c r="DA4" s="54"/>
-      <c r="DB4" s="55"/>
+      <c r="CW4" s="73"/>
+      <c r="CX4" s="73"/>
+      <c r="CY4" s="73"/>
+      <c r="CZ4" s="73"/>
+      <c r="DA4" s="73"/>
+      <c r="DB4" s="74"/>
     </row>
     <row r="5" spans="1:106" ht="15" customHeight="1">
       <c r="A5" s="17" t="s">
@@ -2858,7 +2718,7 @@
       <c r="A8" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="76" t="s">
+      <c r="B8" s="54" t="s">
         <v>40</v>
       </c>
       <c r="C8" s="24" t="s">
@@ -2867,7 +2727,7 @@
       <c r="D8" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="E8" s="77">
+      <c r="E8" s="55">
         <f>Project_Start</f>
         <v>45658</v>
       </c>
@@ -2983,7 +2843,7 @@
       <c r="A9" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="75" t="s">
+      <c r="B9" s="53" t="s">
         <v>34</v>
       </c>
       <c r="C9" s="29" t="s">
@@ -3106,7 +2966,7 @@
       <c r="A10" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="75" t="s">
+      <c r="B10" s="53" t="s">
         <v>35</v>
       </c>
       <c r="C10" s="46" t="s">
@@ -3227,7 +3087,7 @@
     </row>
     <row r="11" spans="1:106" s="13" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A11" s="49"/>
-      <c r="B11" s="75" t="s">
+      <c r="B11" s="53" t="s">
         <v>36</v>
       </c>
       <c r="C11" s="50" t="s">
@@ -3348,11 +3208,11 @@
     </row>
     <row r="12" spans="1:106" s="13" customFormat="1" ht="44" customHeight="1" thickBot="1">
       <c r="A12" s="32"/>
-      <c r="B12" s="75" t="s">
+      <c r="B12" s="53" t="s">
         <v>37</v>
       </c>
       <c r="C12" s="46" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D12" s="30"/>
       <c r="E12" s="31">
@@ -3469,11 +3329,11 @@
     </row>
     <row r="13" spans="1:106" s="13" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A13" s="32"/>
-      <c r="B13" s="75" t="s">
+      <c r="B13" s="53" t="s">
         <v>38</v>
       </c>
       <c r="C13" s="29" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D13" s="30"/>
       <c r="E13" s="31">
@@ -3481,7 +3341,7 @@
         <v>45713</v>
       </c>
       <c r="F13" s="31">
-        <f t="shared" ref="F13:F14" si="7">E13+14</f>
+        <f t="shared" ref="F13" si="7">E13+14</f>
         <v>45727</v>
       </c>
       <c r="G13" s="27"/>
@@ -3592,11 +3452,11 @@
       <c r="A14" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="75" t="s">
+      <c r="B14" s="53" t="s">
         <v>39</v>
       </c>
       <c r="C14" s="48" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D14" s="47"/>
       <c r="E14" s="31">
@@ -3720,17 +3580,6 @@
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="B1:F1"/>
-    <mergeCell ref="B2:F2"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="E3:F3"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="I4:O4"/>
-    <mergeCell ref="P4:V4"/>
-    <mergeCell ref="W4:AC4"/>
-    <mergeCell ref="AD4:AJ4"/>
-    <mergeCell ref="AK4:AQ4"/>
     <mergeCell ref="CH4:CN4"/>
     <mergeCell ref="CO4:CU4"/>
     <mergeCell ref="CV4:DB4"/>
@@ -3740,9 +3589,20 @@
     <mergeCell ref="BM4:BS4"/>
     <mergeCell ref="BT4:BZ4"/>
     <mergeCell ref="CA4:CG4"/>
+    <mergeCell ref="I4:O4"/>
+    <mergeCell ref="P4:V4"/>
+    <mergeCell ref="W4:AC4"/>
+    <mergeCell ref="AD4:AJ4"/>
+    <mergeCell ref="AK4:AQ4"/>
+    <mergeCell ref="B1:F1"/>
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="E4:F4"/>
   </mergeCells>
   <conditionalFormatting sqref="I5:BL14 BM6:DA14 BN5:DA5">
-    <cfRule type="expression" dxfId="21" priority="2">
+    <cfRule type="expression" dxfId="6" priority="2">
       <formula>AND(TODAY()&gt;=I$5,TODAY()&lt;J$5)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3761,28 +3621,28 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BM5">
-    <cfRule type="expression" dxfId="13" priority="8">
+    <cfRule type="expression" dxfId="5" priority="8">
       <formula>AND(TODAY()&gt;=BM$5,TODAY()&lt;BN$5)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I7:DA14">
-    <cfRule type="expression" dxfId="12" priority="56">
+    <cfRule type="expression" dxfId="4" priority="56">
       <formula>AND(task_start&lt;=I$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=I$5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="11" priority="57" stopIfTrue="1">
+    <cfRule type="expression" dxfId="3" priority="57" stopIfTrue="1">
       <formula>AND(task_end&gt;=I$5,task_start&lt;J$5)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="DB5:DB14">
-    <cfRule type="expression" dxfId="5" priority="64">
+    <cfRule type="expression" dxfId="2" priority="64">
       <formula>AND(TODAY()&gt;=DB$5,TODAY()&lt;#REF!)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="DB7:DB14">
-    <cfRule type="expression" dxfId="4" priority="73">
+    <cfRule type="expression" dxfId="1" priority="73">
       <formula>AND(task_start&lt;=DB$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=DB$5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="74" stopIfTrue="1">
+    <cfRule type="expression" dxfId="0" priority="74" stopIfTrue="1">
       <formula>AND(task_end&gt;=DB$5,task_start&lt;#REF!)</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>